<commit_message>
Auto update excel file
</commit_message>
<xml_diff>
--- a/all_grants.xlsx
+++ b/all_grants.xlsx
@@ -609,54 +609,54 @@
 View more featured non-profit jobs
 Latest NGO Jobs
 Post your highlighted jobs here
-Cluster Coordinators
+Account Person
+Sangini
+Location:
+Madhya Pradesh
+Apply by:
+05 Oct 2026
+HR Coordinator
 (Value Members only)
 Location:
-Rajasthan, Gujarat, Maharashtra
+Assam
+Apply by:
+09 Oct 2026
+Counselor
+Asian Minority Action Network
+Location:
+Jharkhand
 Apply by:
 10 Oct 2026
-Computer Instructor
-Help for Children in Need Foundation
-Location:
-Maharashtra
-Apply by:
-30 Sep 2026
-Project Associate
+Master Trainer
 (Value Members only)
 Location:
-Maharashtra
+Gujarat
+Apply by:
+10 Oct 2026
+MIS Executive - DDU-GKY Project
+Nifa India
+Location:
+West Bengal
+Apply by:
+24 Oct 2026
+Fundraising Executive / Manager
+(Value Members only)
+Location:
+Karnataka
 Apply by:
 07 Oct 2026
-Field Coordinator
-Adhwana Kerala Forum of Partners in Functional Vo...
-Location:
-Kerala
-Apply by:
-30 Sep 2026
-Chief Executive Officer
+Community Outreach Workers
+Sangini
+Location:
+Madhya Pradesh
+Apply by:
+05 Oct 2026
+Senior Program Manager, Assistant Project Manager...
 (Value Members only)
 Location:
-Delhi
-Apply by:
-06 Oct 2026
-Support Teacher
-Help for Children in Need Foundation
-Location:
-Maharashtra
-Apply by:
-30 Sep 2026
-Program Manager
-(Value Members only)
-Location:
-West Bengal
-Apply by:
-30 Sep 2026
-Counsellor
-Aditya Information Management Society
-Location:
-Madhya Pradesh
-Apply by:
-30 Sep 2026
+Haryana
+Apply by:
+10 Oct 2026
 View all the latest non-profit jobs
 Jobseekers
 Register
@@ -698,7 +698,7 @@
         </is>
       </c>
       <c r="H2" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I2" s="1" t="inlineStr">
         <is>
@@ -821,54 +821,54 @@
 View more featured non-profit jobs
 Latest NGO Jobs
 Post your highlighted jobs here
-Cluster Coordinators
+Account Person
+Sangini
+Location:
+Madhya Pradesh
+Apply by:
+05 Oct 2026
+HR Coordinator
 (Value Members only)
 Location:
-Rajasthan, Gujarat, Maharashtra
+Assam
+Apply by:
+09 Oct 2026
+Counselor
+Asian Minority Action Network
+Location:
+Jharkhand
 Apply by:
 10 Oct 2026
-Computer Instructor
-Help for Children in Need Foundation
-Location:
-Maharashtra
-Apply by:
-30 Sep 2026
-Project Associate
+Master Trainer
 (Value Members only)
 Location:
-Maharashtra
+Gujarat
+Apply by:
+10 Oct 2026
+MIS Executive - DDU-GKY Project
+Nifa India
+Location:
+West Bengal
+Apply by:
+24 Oct 2026
+Fundraising Executive / Manager
+(Value Members only)
+Location:
+Karnataka
 Apply by:
 07 Oct 2026
-Field Coordinator
-Adhwana Kerala Forum of Partners in Functional Vo...
-Location:
-Kerala
-Apply by:
-30 Sep 2026
-Chief Executive Officer
+Community Outreach Workers
+Sangini
+Location:
+Madhya Pradesh
+Apply by:
+05 Oct 2026
+Senior Program Manager, Assistant Project Manager...
 (Value Members only)
 Location:
-Delhi
-Apply by:
-06 Oct 2026
-Support Teacher
-Help for Children in Need Foundation
-Location:
-Maharashtra
-Apply by:
-30 Sep 2026
-Program Manager
-(Value Members only)
-Location:
-West Bengal
-Apply by:
-30 Sep 2026
-Counsellor
-Aditya Information Management Society
-Location:
-Madhya Pradesh
-Apply by:
-30 Sep 2026
+Haryana
+Apply by:
+10 Oct 2026
 View all the latest non-profit jobs
 Jobseekers
 Register
@@ -910,7 +910,7 @@
         </is>
       </c>
       <c r="H3" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I3" s="1" t="inlineStr">
         <is>
@@ -1078,54 +1078,54 @@
 View more featured non-profit jobs
 Latest NGO Jobs
 Post your highlighted jobs here
-Cluster Coordinators
+Account Person
+Sangini
+Location:
+Madhya Pradesh
+Apply by:
+05 Oct 2026
+HR Coordinator
 (Value Members only)
 Location:
-Rajasthan, Gujarat, Maharashtra
+Assam
+Apply by:
+09 Oct 2026
+Counselor
+Asian Minority Action Network
+Location:
+Jharkhand
 Apply by:
 10 Oct 2026
-Computer Instructor
-Help for Children in Need Foundation
-Location:
-Maharashtra
-Apply by:
-30 Sep 2026
-Project Associate
+Master Trainer
 (Value Members only)
 Location:
-Maharashtra
+Gujarat
+Apply by:
+10 Oct 2026
+MIS Executive - DDU-GKY Project
+Nifa India
+Location:
+West Bengal
+Apply by:
+24 Oct 2026
+Fundraising Executive / Manager
+(Value Members only)
+Location:
+Karnataka
 Apply by:
 07 Oct 2026
-Field Coordinator
-Adhwana Kerala Forum of Partners in Functional Vo...
-Location:
-Kerala
-Apply by:
-30 Sep 2026
-Chief Executive Officer
+Community Outreach Workers
+Sangini
+Location:
+Madhya Pradesh
+Apply by:
+05 Oct 2026
+Senior Program Manager, Assistant Project Manager...
 (Value Members only)
 Location:
-Delhi
-Apply by:
-06 Oct 2026
-Support Teacher
-Help for Children in Need Foundation
-Location:
-Maharashtra
-Apply by:
-30 Sep 2026
-Program Manager
-(Value Members only)
-Location:
-West Bengal
-Apply by:
-30 Sep 2026
-Counsellor
-Aditya Information Management Society
-Location:
-Madhya Pradesh
-Apply by:
-30 Sep 2026
+Haryana
+Apply by:
+10 Oct 2026
 View all the latest non-profit jobs
 Jobseekers
 Register
@@ -1167,7 +1167,7 @@
         </is>
       </c>
       <c r="H4" s="1" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I4" s="1" t="inlineStr">
         <is>
@@ -1304,54 +1304,54 @@
 View more featured non-profit jobs
 Latest NGO Jobs
 Post your highlighted jobs here
-Cluster Coordinators
+Account Person
+Sangini
+Location:
+Madhya Pradesh
+Apply by:
+05 Oct 2026
+HR Coordinator
 (Value Members only)
 Location:
-Rajasthan, Gujarat, Maharashtra
+Assam
+Apply by:
+09 Oct 2026
+Counselor
+Asian Minority Action Network
+Location:
+Jharkhand
 Apply by:
 10 Oct 2026
-Computer Instructor
-Help for Children in Need Foundation
-Location:
-Maharashtra
-Apply by:
-30 Sep 2026
-Project Associate
+Master Trainer
 (Value Members only)
 Location:
-Maharashtra
+Gujarat
+Apply by:
+10 Oct 2026
+MIS Executive - DDU-GKY Project
+Nifa India
+Location:
+West Bengal
+Apply by:
+24 Oct 2026
+Fundraising Executive / Manager
+(Value Members only)
+Location:
+Karnataka
 Apply by:
 07 Oct 2026
-Field Coordinator
-Adhwana Kerala Forum of Partners in Functional Vo...
-Location:
-Kerala
-Apply by:
-30 Sep 2026
-Chief Executive Officer
+Community Outreach Workers
+Sangini
+Location:
+Madhya Pradesh
+Apply by:
+05 Oct 2026
+Senior Program Manager, Assistant Project Manager...
 (Value Members only)
 Location:
-Delhi
-Apply by:
-06 Oct 2026
-Support Teacher
-Help for Children in Need Foundation
-Location:
-Maharashtra
-Apply by:
-30 Sep 2026
-Program Manager
-(Value Members only)
-Location:
-West Bengal
-Apply by:
-30 Sep 2026
-Counsellor
-Aditya Information Management Society
-Location:
-Madhya Pradesh
-Apply by:
-30 Sep 2026
+Haryana
+Apply by:
+10 Oct 2026
 View all the latest non-profit jobs
 Jobseekers
 Register
@@ -1393,7 +1393,7 @@
         </is>
       </c>
       <c r="H5" s="1" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I5" s="1" t="inlineStr">
         <is>
@@ -1549,54 +1549,54 @@
 View more featured non-profit jobs
 Latest NGO Jobs
 Post your highlighted jobs here
-Cluster Coordinators
+Account Person
+Sangini
+Location:
+Madhya Pradesh
+Apply by:
+05 Oct 2026
+HR Coordinator
 (Value Members only)
 Location:
-Rajasthan, Gujarat, Maharashtra
+Assam
+Apply by:
+09 Oct 2026
+Counselor
+Asian Minority Action Network
+Location:
+Jharkhand
 Apply by:
 10 Oct 2026
-Computer Instructor
-Help for Children in Need Foundation
-Location:
-Maharashtra
-Apply by:
-30 Sep 2026
-Project Associate
+Master Trainer
 (Value Members only)
 Location:
-Maharashtra
+Gujarat
+Apply by:
+10 Oct 2026
+MIS Executive - DDU-GKY Project
+Nifa India
+Location:
+West Bengal
+Apply by:
+24 Oct 2026
+Fundraising Executive / Manager
+(Value Members only)
+Location:
+Karnataka
 Apply by:
 07 Oct 2026
-Field Coordinator
-Adhwana Kerala Forum of Partners in Functional Vo...
-Location:
-Kerala
-Apply by:
-30 Sep 2026
-Chief Executive Officer
+Community Outreach Workers
+Sangini
+Location:
+Madhya Pradesh
+Apply by:
+05 Oct 2026
+Senior Program Manager, Assistant Project Manager...
 (Value Members only)
 Location:
-Delhi
-Apply by:
-06 Oct 2026
-Support Teacher
-Help for Children in Need Foundation
-Location:
-Maharashtra
-Apply by:
-30 Sep 2026
-Program Manager
-(Value Members only)
-Location:
-West Bengal
-Apply by:
-30 Sep 2026
-Counsellor
-Aditya Information Management Society
-Location:
-Madhya Pradesh
-Apply by:
-30 Sep 2026
+Haryana
+Apply by:
+10 Oct 2026
 View all the latest non-profit jobs
 Jobseekers
 Register
@@ -1638,7 +1638,7 @@
         </is>
       </c>
       <c r="H6" s="1" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I6" s="1" t="inlineStr">
         <is>
@@ -1812,54 +1812,54 @@
 View more featured non-profit jobs
 Latest NGO Jobs
 Post your highlighted jobs here
-Cluster Coordinators
+Account Person
+Sangini
+Location:
+Madhya Pradesh
+Apply by:
+05 Oct 2026
+HR Coordinator
 (Value Members only)
 Location:
-Rajasthan, Gujarat, Maharashtra
+Assam
+Apply by:
+09 Oct 2026
+Counselor
+Asian Minority Action Network
+Location:
+Jharkhand
 Apply by:
 10 Oct 2026
-Computer Instructor
-Help for Children in Need Foundation
-Location:
-Maharashtra
-Apply by:
-30 Sep 2026
-Project Associate
+Master Trainer
 (Value Members only)
 Location:
-Maharashtra
+Gujarat
+Apply by:
+10 Oct 2026
+MIS Executive - DDU-GKY Project
+Nifa India
+Location:
+West Bengal
+Apply by:
+24 Oct 2026
+Fundraising Executive / Manager
+(Value Members only)
+Location:
+Karnataka
 Apply by:
 07 Oct 2026
-Field Coordinator
-Adhwana Kerala Forum of Partners in Functional Vo...
-Location:
-Kerala
-Apply by:
-30 Sep 2026
-Chief Executive Officer
+Community Outreach Workers
+Sangini
+Location:
+Madhya Pradesh
+Apply by:
+05 Oct 2026
+Senior Program Manager, Assistant Project Manager...
 (Value Members only)
 Location:
-Delhi
-Apply by:
-06 Oct 2026
-Support Teacher
-Help for Children in Need Foundation
-Location:
-Maharashtra
-Apply by:
-30 Sep 2026
-Program Manager
-(Value Members only)
-Location:
-West Bengal
-Apply by:
-30 Sep 2026
-Counsellor
-Aditya Information Management Society
-Location:
-Madhya Pradesh
-Apply by:
-30 Sep 2026
+Haryana
+Apply by:
+10 Oct 2026
 View all the latest non-profit jobs
 Jobseekers
 Register
@@ -1901,7 +1901,7 @@
         </is>
       </c>
       <c r="H7" s="1" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I7" s="1" t="inlineStr">
         <is>
@@ -1946,7 +1946,7 @@
         </is>
       </c>
       <c r="H8" s="1" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I8" s="1" t="inlineStr">
         <is>
@@ -1991,7 +1991,7 @@
         </is>
       </c>
       <c r="H9" s="1" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I9" s="1" t="inlineStr">
         <is>
@@ -2036,7 +2036,7 @@
         </is>
       </c>
       <c r="H10" s="1" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I10" s="1" t="inlineStr">
         <is>
@@ -2081,7 +2081,7 @@
         </is>
       </c>
       <c r="H11" s="1" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I11" s="1" t="inlineStr">
         <is>
@@ -2126,7 +2126,7 @@
         </is>
       </c>
       <c r="H12" s="1" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I12" s="1" t="inlineStr">
         <is>
@@ -2171,7 +2171,7 @@
         </is>
       </c>
       <c r="H13" s="1" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I13" s="1" t="inlineStr">
         <is>
@@ -2216,7 +2216,7 @@
         </is>
       </c>
       <c r="H14" s="1" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I14" s="1" t="inlineStr">
         <is>
@@ -2261,7 +2261,7 @@
         </is>
       </c>
       <c r="H15" s="1" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I15" s="1" t="inlineStr">
         <is>
@@ -2310,7 +2310,7 @@
         </is>
       </c>
       <c r="H16" s="1" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I16" s="1" t="inlineStr">
         <is>
@@ -2355,7 +2355,7 @@
         </is>
       </c>
       <c r="H17" s="1" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I17" s="1" t="inlineStr">
         <is>
@@ -2400,7 +2400,7 @@
         </is>
       </c>
       <c r="H18" s="1" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I18" s="1" t="inlineStr">
         <is>
@@ -2606,54 +2606,54 @@
 View more featured non-profit jobs
 Latest NGO Jobs
 Post your highlighted jobs here
-Cluster Coordinators
+Account Person
+Sangini
+Location:
+Madhya Pradesh
+Apply by:
+05 Oct 2026
+HR Coordinator
 (Value Members only)
 Location:
-Rajasthan, Gujarat, Maharashtra
+Assam
+Apply by:
+09 Oct 2026
+Counselor
+Asian Minority Action Network
+Location:
+Jharkhand
 Apply by:
 10 Oct 2026
-Computer Instructor
-Help for Children in Need Foundation
-Location:
-Maharashtra
-Apply by:
-30 Sep 2026
-Project Associate
+Master Trainer
 (Value Members only)
 Location:
-Maharashtra
+Gujarat
+Apply by:
+10 Oct 2026
+MIS Executive - DDU-GKY Project
+Nifa India
+Location:
+West Bengal
+Apply by:
+24 Oct 2026
+Fundraising Executive / Manager
+(Value Members only)
+Location:
+Karnataka
 Apply by:
 07 Oct 2026
-Field Coordinator
-Adhwana Kerala Forum of Partners in Functional Vo...
-Location:
-Kerala
-Apply by:
-30 Sep 2026
-Chief Executive Officer
+Community Outreach Workers
+Sangini
+Location:
+Madhya Pradesh
+Apply by:
+05 Oct 2026
+Senior Program Manager, Assistant Project Manager...
 (Value Members only)
 Location:
-Delhi
-Apply by:
-06 Oct 2026
-Support Teacher
-Help for Children in Need Foundation
-Location:
-Maharashtra
-Apply by:
-30 Sep 2026
-Program Manager
-(Value Members only)
-Location:
-West Bengal
-Apply by:
-30 Sep 2026
-Counsellor
-Aditya Information Management Society
-Location:
-Madhya Pradesh
-Apply by:
-30 Sep 2026
+Haryana
+Apply by:
+10 Oct 2026
 View all the latest non-profit jobs
 Jobseekers
 Register
@@ -2695,7 +2695,7 @@
         </is>
       </c>
       <c r="H19" s="1" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I19" s="1" t="inlineStr">
         <is>
@@ -2740,7 +2740,7 @@
         </is>
       </c>
       <c r="H20" s="1" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I20" s="1" t="inlineStr">
         <is>
@@ -2785,7 +2785,7 @@
         </is>
       </c>
       <c r="H21" s="1" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I21" s="1" t="inlineStr">
         <is>
@@ -2830,7 +2830,7 @@
         </is>
       </c>
       <c r="H22" s="1" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I22" s="1" t="inlineStr">
         <is>
@@ -3006,54 +3006,54 @@
 View more featured non-profit jobs
 Latest NGO Jobs
 Post your highlighted jobs here
-Cluster Coordinators
+Account Person
+Sangini
+Location:
+Madhya Pradesh
+Apply by:
+05 Oct 2026
+HR Coordinator
 (Value Members only)
 Location:
-Rajasthan, Gujarat, Maharashtra
+Assam
+Apply by:
+09 Oct 2026
+Counselor
+Asian Minority Action Network
+Location:
+Jharkhand
 Apply by:
 10 Oct 2026
-Computer Instructor
-Help for Children in Need Foundation
-Location:
-Maharashtra
-Apply by:
-30 Sep 2026
-Project Associate
+Master Trainer
 (Value Members only)
 Location:
-Maharashtra
+Gujarat
+Apply by:
+10 Oct 2026
+MIS Executive - DDU-GKY Project
+Nifa India
+Location:
+West Bengal
+Apply by:
+24 Oct 2026
+Fundraising Executive / Manager
+(Value Members only)
+Location:
+Karnataka
 Apply by:
 07 Oct 2026
-Field Coordinator
-Adhwana Kerala Forum of Partners in Functional Vo...
-Location:
-Kerala
-Apply by:
-30 Sep 2026
-Chief Executive Officer
+Community Outreach Workers
+Sangini
+Location:
+Madhya Pradesh
+Apply by:
+05 Oct 2026
+Senior Program Manager, Assistant Project Manager...
 (Value Members only)
 Location:
-Delhi
-Apply by:
-06 Oct 2026
-Support Teacher
-Help for Children in Need Foundation
-Location:
-Maharashtra
-Apply by:
-30 Sep 2026
-Program Manager
-(Value Members only)
-Location:
-West Bengal
-Apply by:
-30 Sep 2026
-Counsellor
-Aditya Information Management Society
-Location:
-Madhya Pradesh
-Apply by:
-30 Sep 2026
+Haryana
+Apply by:
+10 Oct 2026
 View all the latest non-profit jobs
 Jobseekers
 Register
@@ -3095,7 +3095,7 @@
         </is>
       </c>
       <c r="H23" s="1" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I23" s="1" t="inlineStr">
         <is>
@@ -3227,54 +3227,54 @@
 View more featured non-profit jobs
 Latest NGO Jobs
 Post your highlighted jobs here
-Cluster Coordinators
+Account Person
+Sangini
+Location:
+Madhya Pradesh
+Apply by:
+05 Oct 2026
+HR Coordinator
 (Value Members only)
 Location:
-Rajasthan, Gujarat, Maharashtra
+Assam
+Apply by:
+09 Oct 2026
+Counselor
+Asian Minority Action Network
+Location:
+Jharkhand
 Apply by:
 10 Oct 2026
-Computer Instructor
-Help for Children in Need Foundation
-Location:
-Maharashtra
-Apply by:
-30 Sep 2026
-Project Associate
+Master Trainer
 (Value Members only)
 Location:
-Maharashtra
+Gujarat
+Apply by:
+10 Oct 2026
+MIS Executive - DDU-GKY Project
+Nifa India
+Location:
+West Bengal
+Apply by:
+24 Oct 2026
+Fundraising Executive / Manager
+(Value Members only)
+Location:
+Karnataka
 Apply by:
 07 Oct 2026
-Field Coordinator
-Adhwana Kerala Forum of Partners in Functional Vo...
-Location:
-Kerala
-Apply by:
-30 Sep 2026
-Chief Executive Officer
+Community Outreach Workers
+Sangini
+Location:
+Madhya Pradesh
+Apply by:
+05 Oct 2026
+Senior Program Manager, Assistant Project Manager...
 (Value Members only)
 Location:
-Delhi
-Apply by:
-06 Oct 2026
-Support Teacher
-Help for Children in Need Foundation
-Location:
-Maharashtra
-Apply by:
-30 Sep 2026
-Program Manager
-(Value Members only)
-Location:
-West Bengal
-Apply by:
-30 Sep 2026
-Counsellor
-Aditya Information Management Society
-Location:
-Madhya Pradesh
-Apply by:
-30 Sep 2026
+Haryana
+Apply by:
+10 Oct 2026
 View all the latest non-profit jobs
 Jobseekers
 Register
@@ -3316,7 +3316,7 @@
         </is>
       </c>
       <c r="H24" s="1" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="I24" s="1" t="inlineStr">
         <is>
@@ -3480,54 +3480,54 @@
 View more featured non-profit jobs
 Latest NGO Jobs
 Post your highlighted jobs here
-Cluster Coordinators
+Account Person
+Sangini
+Location:
+Madhya Pradesh
+Apply by:
+05 Oct 2026
+HR Coordinator
 (Value Members only)
 Location:
-Rajasthan, Gujarat, Maharashtra
+Assam
+Apply by:
+09 Oct 2026
+Counselor
+Asian Minority Action Network
+Location:
+Jharkhand
 Apply by:
 10 Oct 2026
-Computer Instructor
-Help for Children in Need Foundation
-Location:
-Maharashtra
-Apply by:
-30 Sep 2026
-Project Associate
+Master Trainer
 (Value Members only)
 Location:
-Maharashtra
+Gujarat
+Apply by:
+10 Oct 2026
+MIS Executive - DDU-GKY Project
+Nifa India
+Location:
+West Bengal
+Apply by:
+24 Oct 2026
+Fundraising Executive / Manager
+(Value Members only)
+Location:
+Karnataka
 Apply by:
 07 Oct 2026
-Field Coordinator
-Adhwana Kerala Forum of Partners in Functional Vo...
-Location:
-Kerala
-Apply by:
-30 Sep 2026
-Chief Executive Officer
+Community Outreach Workers
+Sangini
+Location:
+Madhya Pradesh
+Apply by:
+05 Oct 2026
+Senior Program Manager, Assistant Project Manager...
 (Value Members only)
 Location:
-Delhi
-Apply by:
-06 Oct 2026
-Support Teacher
-Help for Children in Need Foundation
-Location:
-Maharashtra
-Apply by:
-30 Sep 2026
-Program Manager
-(Value Members only)
-Location:
-West Bengal
-Apply by:
-30 Sep 2026
-Counsellor
-Aditya Information Management Society
-Location:
-Madhya Pradesh
-Apply by:
-30 Sep 2026
+Haryana
+Apply by:
+10 Oct 2026
 View all the latest non-profit jobs
 Jobseekers
 Register
@@ -3569,7 +3569,7 @@
         </is>
       </c>
       <c r="H25" s="1" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="I25" s="1" t="inlineStr">
         <is>
@@ -3695,54 +3695,54 @@
 View more featured non-profit jobs
 Latest NGO Jobs
 Post your highlighted jobs here
-Cluster Coordinators
+Account Person
+Sangini
+Location:
+Madhya Pradesh
+Apply by:
+05 Oct 2026
+HR Coordinator
 (Value Members only)
 Location:
-Rajasthan, Gujarat, Maharashtra
+Assam
+Apply by:
+09 Oct 2026
+Counselor
+Asian Minority Action Network
+Location:
+Jharkhand
 Apply by:
 10 Oct 2026
-Computer Instructor
-Help for Children in Need Foundation
-Location:
-Maharashtra
-Apply by:
-30 Sep 2026
-Project Associate
+Master Trainer
 (Value Members only)
 Location:
-Maharashtra
+Gujarat
+Apply by:
+10 Oct 2026
+MIS Executive - DDU-GKY Project
+Nifa India
+Location:
+West Bengal
+Apply by:
+24 Oct 2026
+Fundraising Executive / Manager
+(Value Members only)
+Location:
+Karnataka
 Apply by:
 07 Oct 2026
-Field Coordinator
-Adhwana Kerala Forum of Partners in Functional Vo...
-Location:
-Kerala
-Apply by:
-30 Sep 2026
-Chief Executive Officer
+Community Outreach Workers
+Sangini
+Location:
+Madhya Pradesh
+Apply by:
+05 Oct 2026
+Senior Program Manager, Assistant Project Manager...
 (Value Members only)
 Location:
-Delhi
-Apply by:
-06 Oct 2026
-Support Teacher
-Help for Children in Need Foundation
-Location:
-Maharashtra
-Apply by:
-30 Sep 2026
-Program Manager
-(Value Members only)
-Location:
-West Bengal
-Apply by:
-30 Sep 2026
-Counsellor
-Aditya Information Management Society
-Location:
-Madhya Pradesh
-Apply by:
-30 Sep 2026
+Haryana
+Apply by:
+10 Oct 2026
 View all the latest non-profit jobs
 Jobseekers
 Register
@@ -3784,7 +3784,7 @@
         </is>
       </c>
       <c r="H26" s="1" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="I26" s="1" t="inlineStr">
         <is>
@@ -3829,7 +3829,7 @@
         </is>
       </c>
       <c r="H27" s="1" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="I27" s="1" t="inlineStr">
         <is>
@@ -3874,7 +3874,7 @@
         </is>
       </c>
       <c r="H28" s="1" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="I28" s="1" t="inlineStr">
         <is>
@@ -3919,7 +3919,7 @@
         </is>
       </c>
       <c r="H29" s="1" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="I29" s="1" t="inlineStr">
         <is>
@@ -3964,7 +3964,7 @@
         </is>
       </c>
       <c r="H30" s="1" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="I30" s="1" t="inlineStr">
         <is>
@@ -4116,54 +4116,54 @@
 View more featured non-profit jobs
 Latest NGO Jobs
 Post your highlighted jobs here
-Cluster Coordinators
+Account Person
+Sangini
+Location:
+Madhya Pradesh
+Apply by:
+05 Oct 2026
+HR Coordinator
 (Value Members only)
 Location:
-Rajasthan, Gujarat, Maharashtra
+Assam
+Apply by:
+09 Oct 2026
+Counselor
+Asian Minority Action Network
+Location:
+Jharkhand
 Apply by:
 10 Oct 2026
-Computer Instructor
-Help for Children in Need Foundation
-Location:
-Maharashtra
-Apply by:
-30 Sep 2026
-Project Associate
+Master Trainer
 (Value Members only)
 Location:
-Maharashtra
+Gujarat
+Apply by:
+10 Oct 2026
+MIS Executive - DDU-GKY Project
+Nifa India
+Location:
+West Bengal
+Apply by:
+24 Oct 2026
+Fundraising Executive / Manager
+(Value Members only)
+Location:
+Karnataka
 Apply by:
 07 Oct 2026
-Field Coordinator
-Adhwana Kerala Forum of Partners in Functional Vo...
-Location:
-Kerala
-Apply by:
-30 Sep 2026
-Chief Executive Officer
+Community Outreach Workers
+Sangini
+Location:
+Madhya Pradesh
+Apply by:
+05 Oct 2026
+Senior Program Manager, Assistant Project Manager...
 (Value Members only)
 Location:
-Delhi
-Apply by:
-06 Oct 2026
-Support Teacher
-Help for Children in Need Foundation
-Location:
-Maharashtra
-Apply by:
-30 Sep 2026
-Program Manager
-(Value Members only)
-Location:
-West Bengal
-Apply by:
-30 Sep 2026
-Counsellor
-Aditya Information Management Society
-Location:
-Madhya Pradesh
-Apply by:
-30 Sep 2026
+Haryana
+Apply by:
+10 Oct 2026
 View all the latest non-profit jobs
 Jobseekers
 Register
@@ -4205,7 +4205,7 @@
         </is>
       </c>
       <c r="H31" s="1" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="I31" s="1" t="inlineStr">
         <is>
@@ -4250,7 +4250,7 @@
         </is>
       </c>
       <c r="H32" s="1" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="I32" s="1" t="inlineStr">
         <is>
@@ -4364,54 +4364,54 @@
 View more featured non-profit jobs
 Latest NGO Jobs
 Post your highlighted jobs here
-Cluster Coordinators
+Account Person
+Sangini
+Location:
+Madhya Pradesh
+Apply by:
+05 Oct 2026
+HR Coordinator
 (Value Members only)
 Location:
-Rajasthan, Gujarat, Maharashtra
+Assam
+Apply by:
+09 Oct 2026
+Counselor
+Asian Minority Action Network
+Location:
+Jharkhand
 Apply by:
 10 Oct 2026
-Computer Instructor
-Help for Children in Need Foundation
-Location:
-Maharashtra
-Apply by:
-30 Sep 2026
-Project Associate
+Master Trainer
 (Value Members only)
 Location:
-Maharashtra
+Gujarat
+Apply by:
+10 Oct 2026
+MIS Executive - DDU-GKY Project
+Nifa India
+Location:
+West Bengal
+Apply by:
+24 Oct 2026
+Fundraising Executive / Manager
+(Value Members only)
+Location:
+Karnataka
 Apply by:
 07 Oct 2026
-Field Coordinator
-Adhwana Kerala Forum of Partners in Functional Vo...
-Location:
-Kerala
-Apply by:
-30 Sep 2026
-Chief Executive Officer
+Community Outreach Workers
+Sangini
+Location:
+Madhya Pradesh
+Apply by:
+05 Oct 2026
+Senior Program Manager, Assistant Project Manager...
 (Value Members only)
 Location:
-Delhi
-Apply by:
-06 Oct 2026
-Support Teacher
-Help for Children in Need Foundation
-Location:
-Maharashtra
-Apply by:
-30 Sep 2026
-Program Manager
-(Value Members only)
-Location:
-West Bengal
-Apply by:
-30 Sep 2026
-Counsellor
-Aditya Information Management Society
-Location:
-Madhya Pradesh
-Apply by:
-30 Sep 2026
+Haryana
+Apply by:
+10 Oct 2026
 View all the latest non-profit jobs
 Jobseekers
 Register
@@ -4453,7 +4453,7 @@
         </is>
       </c>
       <c r="H33" s="1" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="I33" s="1" t="inlineStr">
         <is>
@@ -4498,7 +4498,7 @@
         </is>
       </c>
       <c r="H34" s="1" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="I34" s="1" t="inlineStr">
         <is>
@@ -4543,7 +4543,7 @@
         </is>
       </c>
       <c r="H35" s="1" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="I35" s="1" t="inlineStr">
         <is>
@@ -4588,7 +4588,7 @@
         </is>
       </c>
       <c r="H36" s="1" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="I36" s="1" t="inlineStr">
         <is>
@@ -4633,7 +4633,7 @@
         </is>
       </c>
       <c r="H37" s="1" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="I37" s="1" t="inlineStr">
         <is>
@@ -4678,7 +4678,7 @@
         </is>
       </c>
       <c r="H38" s="1" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="I38" s="1" t="inlineStr">
         <is>
@@ -4723,7 +4723,7 @@
         </is>
       </c>
       <c r="H39" s="1" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="I39" s="1" t="inlineStr">
         <is>
@@ -4768,7 +4768,7 @@
         </is>
       </c>
       <c r="H40" s="1" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="I40" s="1" t="inlineStr">
         <is>
@@ -4813,7 +4813,7 @@
         </is>
       </c>
       <c r="H41" s="1" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="I41" s="1" t="inlineStr">
         <is>
@@ -4858,7 +4858,7 @@
         </is>
       </c>
       <c r="H42" s="1" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="I42" s="1" t="inlineStr">
         <is>
@@ -4903,7 +4903,7 @@
         </is>
       </c>
       <c r="H43" s="1" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="I43" s="1" t="inlineStr">
         <is>
@@ -4948,7 +4948,7 @@
         </is>
       </c>
       <c r="H44" s="1" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="I44" s="1" t="inlineStr">
         <is>
@@ -4993,7 +4993,7 @@
         </is>
       </c>
       <c r="H45" s="1" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="I45" s="1" t="inlineStr">
         <is>
@@ -5038,7 +5038,7 @@
         </is>
       </c>
       <c r="H46" s="1" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="I46" s="1" t="inlineStr">
         <is>
@@ -5083,7 +5083,7 @@
         </is>
       </c>
       <c r="H47" s="1" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="I47" s="1" t="inlineStr">
         <is>
@@ -5128,7 +5128,7 @@
         </is>
       </c>
       <c r="H48" s="1" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="I48" s="1" t="inlineStr">
         <is>
@@ -5173,7 +5173,7 @@
         </is>
       </c>
       <c r="H49" s="1" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="I49" s="1" t="inlineStr">
         <is>
@@ -5218,7 +5218,7 @@
         </is>
       </c>
       <c r="H50" s="1" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="I50" s="1" t="inlineStr">
         <is>
@@ -5376,54 +5376,54 @@
 View more featured non-profit jobs
 Latest NGO Jobs
 Post your highlighted jobs here
-Cluster Coordinators
+Account Person
+Sangini
+Location:
+Madhya Pradesh
+Apply by:
+05 Oct 2026
+HR Coordinator
 (Value Members only)
 Location:
-Rajasthan, Gujarat, Maharashtra
+Assam
+Apply by:
+09 Oct 2026
+Counselor
+Asian Minority Action Network
+Location:
+Jharkhand
 Apply by:
 10 Oct 2026
-Computer Instructor
-Help for Children in Need Foundation
-Location:
-Maharashtra
-Apply by:
-30 Sep 2026
-Project Associate
+Master Trainer
 (Value Members only)
 Location:
-Maharashtra
+Gujarat
+Apply by:
+10 Oct 2026
+MIS Executive - DDU-GKY Project
+Nifa India
+Location:
+West Bengal
+Apply by:
+24 Oct 2026
+Fundraising Executive / Manager
+(Value Members only)
+Location:
+Karnataka
 Apply by:
 07 Oct 2026
-Field Coordinator
-Adhwana Kerala Forum of Partners in Functional Vo...
-Location:
-Kerala
-Apply by:
-30 Sep 2026
-Chief Executive Officer
+Community Outreach Workers
+Sangini
+Location:
+Madhya Pradesh
+Apply by:
+05 Oct 2026
+Senior Program Manager, Assistant Project Manager...
 (Value Members only)
 Location:
-Delhi
-Apply by:
-06 Oct 2026
-Support Teacher
-Help for Children in Need Foundation
-Location:
-Maharashtra
-Apply by:
-30 Sep 2026
-Program Manager
-(Value Members only)
-Location:
-West Bengal
-Apply by:
-30 Sep 2026
-Counsellor
-Aditya Information Management Society
-Location:
-Madhya Pradesh
-Apply by:
-30 Sep 2026
+Haryana
+Apply by:
+10 Oct 2026
 View all the latest non-profit jobs
 Jobseekers
 Register
@@ -5465,7 +5465,7 @@
         </is>
       </c>
       <c r="H51" s="1" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="I51" s="1" t="inlineStr">
         <is>
@@ -5510,7 +5510,7 @@
         </is>
       </c>
       <c r="H52" s="1" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="I52" s="1" t="inlineStr">
         <is>
@@ -5555,7 +5555,7 @@
         </is>
       </c>
       <c r="H53" s="1" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="I53" s="1" t="inlineStr">
         <is>
@@ -5600,7 +5600,7 @@
         </is>
       </c>
       <c r="H54" s="1" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="I54" s="1" t="inlineStr">
         <is>
@@ -5645,7 +5645,7 @@
         </is>
       </c>
       <c r="H55" s="1" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="I55" s="1" t="inlineStr">
         <is>
@@ -5690,7 +5690,7 @@
         </is>
       </c>
       <c r="H56" s="1" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="I56" s="1" t="inlineStr">
         <is>
@@ -5735,7 +5735,7 @@
         </is>
       </c>
       <c r="H57" s="1" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="I57" s="1" t="inlineStr">
         <is>
@@ -5780,7 +5780,7 @@
         </is>
       </c>
       <c r="H58" s="1" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="I58" s="1" t="inlineStr">
         <is>
@@ -5825,7 +5825,7 @@
         </is>
       </c>
       <c r="H59" s="1" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="I59" s="1" t="inlineStr">
         <is>
@@ -5870,7 +5870,7 @@
         </is>
       </c>
       <c r="H60" s="1" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="I60" s="1" t="inlineStr">
         <is>
@@ -5915,7 +5915,7 @@
         </is>
       </c>
       <c r="H61" s="1" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="I61" s="1" t="inlineStr">
         <is>
@@ -5960,7 +5960,7 @@
         </is>
       </c>
       <c r="H62" s="1" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="I62" s="1" t="inlineStr">
         <is>
@@ -6005,7 +6005,7 @@
         </is>
       </c>
       <c r="H63" s="1" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="I63" s="1" t="inlineStr">
         <is>
@@ -6050,7 +6050,7 @@
         </is>
       </c>
       <c r="H64" s="1" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="I64" s="1" t="inlineStr">
         <is>
@@ -6161,54 +6161,54 @@
 View more featured non-profit jobs
 Latest NGO Jobs
 Post your highlighted jobs here
-Cluster Coordinators
+Account Person
+Sangini
+Location:
+Madhya Pradesh
+Apply by:
+05 Oct 2026
+HR Coordinator
 (Value Members only)
 Location:
-Rajasthan, Gujarat, Maharashtra
+Assam
+Apply by:
+09 Oct 2026
+Counselor
+Asian Minority Action Network
+Location:
+Jharkhand
 Apply by:
 10 Oct 2026
-Computer Instructor
-Help for Children in Need Foundation
-Location:
-Maharashtra
-Apply by:
-30 Sep 2026
-Project Associate
+Master Trainer
 (Value Members only)
 Location:
-Maharashtra
+Gujarat
+Apply by:
+10 Oct 2026
+MIS Executive - DDU-GKY Project
+Nifa India
+Location:
+West Bengal
+Apply by:
+24 Oct 2026
+Fundraising Executive / Manager
+(Value Members only)
+Location:
+Karnataka
 Apply by:
 07 Oct 2026
-Field Coordinator
-Adhwana Kerala Forum of Partners in Functional Vo...
-Location:
-Kerala
-Apply by:
-30 Sep 2026
-Chief Executive Officer
+Community Outreach Workers
+Sangini
+Location:
+Madhya Pradesh
+Apply by:
+05 Oct 2026
+Senior Program Manager, Assistant Project Manager...
 (Value Members only)
 Location:
-Delhi
-Apply by:
-06 Oct 2026
-Support Teacher
-Help for Children in Need Foundation
-Location:
-Maharashtra
-Apply by:
-30 Sep 2026
-Program Manager
-(Value Members only)
-Location:
-West Bengal
-Apply by:
-30 Sep 2026
-Counsellor
-Aditya Information Management Society
-Location:
-Madhya Pradesh
-Apply by:
-30 Sep 2026
+Haryana
+Apply by:
+10 Oct 2026
 View all the latest non-profit jobs
 Jobseekers
 Register
@@ -6250,7 +6250,7 @@
         </is>
       </c>
       <c r="H65" s="1" t="n">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="I65" s="1" t="inlineStr">
         <is>
@@ -6295,7 +6295,7 @@
         </is>
       </c>
       <c r="H66" s="1" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="I66" s="1" t="inlineStr">
         <is>
@@ -6340,7 +6340,7 @@
         </is>
       </c>
       <c r="H67" s="1" t="n">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="I67" s="1" t="inlineStr">
         <is>
@@ -6385,7 +6385,7 @@
         </is>
       </c>
       <c r="H68" s="1" t="n">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="I68" s="1" t="inlineStr">
         <is>
@@ -6430,7 +6430,7 @@
         </is>
       </c>
       <c r="H69" s="1" t="n">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="I69" s="1" t="inlineStr">
         <is>
@@ -6475,7 +6475,7 @@
         </is>
       </c>
       <c r="H70" s="1" t="n">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="I70" s="1" t="inlineStr">
         <is>
@@ -6520,7 +6520,7 @@
         </is>
       </c>
       <c r="H71" s="1" t="n">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="I71" s="1" t="inlineStr">
         <is>
@@ -6565,7 +6565,7 @@
         </is>
       </c>
       <c r="H72" s="1" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="I72" s="1" t="inlineStr">
         <is>
@@ -6610,7 +6610,7 @@
         </is>
       </c>
       <c r="H73" s="1" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="I73" s="1" t="inlineStr">
         <is>
@@ -6655,7 +6655,7 @@
         </is>
       </c>
       <c r="H74" s="1" t="n">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="I74" s="1" t="inlineStr">
         <is>
@@ -6700,7 +6700,7 @@
         </is>
       </c>
       <c r="H75" s="1" t="n">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="I75" s="1" t="inlineStr">
         <is>
@@ -6745,7 +6745,7 @@
         </is>
       </c>
       <c r="H76" s="1" t="n">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="I76" s="1" t="inlineStr">
         <is>
@@ -6790,7 +6790,7 @@
         </is>
       </c>
       <c r="H77" s="1" t="n">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="I77" s="1" t="inlineStr">
         <is>
@@ -6835,7 +6835,7 @@
         </is>
       </c>
       <c r="H78" s="1" t="n">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="I78" s="1" t="inlineStr">
         <is>
@@ -6880,7 +6880,7 @@
         </is>
       </c>
       <c r="H79" s="1" t="n">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="I79" s="1" t="inlineStr">
         <is>
@@ -6925,7 +6925,7 @@
         </is>
       </c>
       <c r="H80" s="1" t="n">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="I80" s="1" t="inlineStr">
         <is>
@@ -6970,7 +6970,7 @@
         </is>
       </c>
       <c r="H81" s="1" t="n">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="I81" s="1" t="inlineStr">
         <is>
@@ -7015,7 +7015,7 @@
         </is>
       </c>
       <c r="H82" s="1" t="n">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="I82" s="1" t="inlineStr">
         <is>
@@ -7060,7 +7060,7 @@
         </is>
       </c>
       <c r="H83" s="1" t="n">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="I83" s="1" t="inlineStr">
         <is>
@@ -7105,7 +7105,7 @@
         </is>
       </c>
       <c r="H84" s="1" t="n">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="I84" s="1" t="inlineStr">
         <is>
@@ -7150,7 +7150,7 @@
         </is>
       </c>
       <c r="H85" s="1" t="n">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="I85" s="1" t="inlineStr">
         <is>
@@ -7195,7 +7195,7 @@
         </is>
       </c>
       <c r="H86" s="1" t="n">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="I86" s="1" t="inlineStr">
         <is>

</xml_diff>